<commit_message>
feat(retina): implement EfficientNet-B0 baseline framework with training pipeline and Volume 4 documentation
</commit_message>
<xml_diff>
--- a/experiments/experiment_log.xlsx
+++ b/experiments/experiment_log.xlsx
@@ -8,24 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\FusionMedAI\experiments\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{200EA883-1832-4AC8-A868-C6FCB2DABD88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F95DFDCE-C4B5-4B72-82E5-DBB174717CC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{BE96C83E-606E-49D3-9661-F42589127FFA}"/>
+    <workbookView xWindow="3276" yWindow="3276" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="41">
   <si>
     <t>ID</t>
   </si>
@@ -130,6 +125,24 @@
   </si>
   <si>
     <t>default</t>
+  </si>
+  <si>
+    <t>2026-06-28</t>
+  </si>
+  <si>
+    <t>efficientnet_b0</t>
+  </si>
+  <si>
+    <t>lr=0.0001, bs=32, size=224</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>Inference Latency: 17.41 ms</t>
+  </si>
+  <si>
+    <t>Completed</t>
   </si>
 </sst>
 </file>
@@ -497,17 +510,17 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF13585D-5E43-4B65-A155-6BD6C422A7FA}">
-  <dimension ref="A1:Q5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:Q6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="12" customWidth="1"/>
-    <col min="4" max="4" width="12.6640625" customWidth="1"/>
-    <col min="6" max="6" width="9.88671875" customWidth="1"/>
-    <col min="7" max="7" width="16.5546875" customWidth="1"/>
+    <col min="2" max="2" width="13.88671875" customWidth="1"/>
+    <col min="4" max="4" width="18.44140625" customWidth="1"/>
+    <col min="6" max="6" width="15.44140625" customWidth="1"/>
+    <col min="7" max="7" width="23.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -560,7 +573,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:17" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:17" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -595,7 +608,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:17" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:17" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -630,7 +643,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:17" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:17" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -665,7 +678,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:17" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:17" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -700,6 +713,59 @@
         <v>22</v>
       </c>
     </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>35</v>
+      </c>
+      <c r="C6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" t="s">
+        <v>36</v>
+      </c>
+      <c r="E6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F6" t="s">
+        <v>36</v>
+      </c>
+      <c r="G6" t="s">
+        <v>37</v>
+      </c>
+      <c r="H6">
+        <v>9.375E-2</v>
+      </c>
+      <c r="I6">
+        <v>2.7272727272727271E-2</v>
+      </c>
+      <c r="J6">
+        <v>0.1</v>
+      </c>
+      <c r="K6">
+        <v>4.2857142857142858E-2</v>
+      </c>
+      <c r="L6">
+        <v>0.50290902334380605</v>
+      </c>
+      <c r="M6" t="s">
+        <v>38</v>
+      </c>
+      <c r="N6" t="s">
+        <v>38</v>
+      </c>
+      <c r="O6" t="s">
+        <v>38</v>
+      </c>
+      <c r="P6" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>40</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>